<commit_message>
Task 4.3: Echo experiment SE trigger points
Adds SE playback calls to the four chapter-2 echo experiment
dramas via resolve_run() on cmd.elinikki.audio.se.play.<id>:

  * stage 1 — footstep echo once at drama open (awareness)
  * stage 2 — two clap+return pairs (mismatched 3s→2s timing)
  * stage 3 — three claps + three returns (count preserved)
  * stage 4 — five claps + one pattern return (PHM climax
              "2→pause→3" cadence)

Shared constants live in elinikki_echo_stage_1.py and are
imported by the other stage scripts. The SE ids themselves
(elinikki_echo_footstep etc.) are provisional placeholders until
Task 6.1 in-game verification picks the actual vanilla Elin
sound assets; PlaySe already logs a Warn when the id does not
resolve, so missing placeholders fail loud without breaking the
drama.

build.bat debug: 0 warnings, 0 errors.
</commit_message>
<xml_diff>
--- a/Elin_Elinikki/LangMod/EN/Dialog/Drama/drama_elinikki_echo_stage_1.xlsx
+++ b/Elin_Elinikki/LangMod/EN/Dialog/Drama/drama_elinikki_echo_stage_1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,30 +539,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>narrator</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>echo1_sora_ceiling</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>ソラ:「天井が……見えない。とんでもない規模だ」</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Sora: 'Can't see the ceiling. The scale of this place...'</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Sora: 'Can't see the ceiling. The scale of this place...'</t>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>eval</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Elin_QuestMod.Drama.DramaRuntime.ResolveRun("cmd.elinikki.audio.se.play.elinikki_echo_footstep");</t>
         </is>
       </c>
     </row>
@@ -574,23 +558,23 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>echo1_mina_watch</t>
+          <t>echo1_sora_ceiling</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>ミナ:「足元見ろ。上向いてると落ちる」</t>
+          <t>ソラ:「天井が……見えない。とんでもない規模だ」</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Mina: 'Eyes down. You'll fall if you keep looking up.'</t>
+          <t>Sora: 'Can't see the ceiling. The scale of this place...'</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Mina: 'Eyes down. You'll fall if you keep looking up.'</t>
+          <t>Sora: 'Can't see the ceiling. The scale of this place...'</t>
         </is>
       </c>
     </row>
@@ -602,23 +586,23 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>echo1_sora_timing</t>
+          <t>echo1_mina_watch</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>ソラ:「……足音の返り、距離と合わないな」</t>
+          <t>ミナ:「足元見ろ。上向いてると落ちる」</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Sora: '...The echo timing. It doesn't match the distance.'</t>
+          <t>Mina: 'Eyes down. You'll fall if you keep looking up.'</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Sora: '...The echo timing. It doesn't match the distance.'</t>
+          <t>Mina: 'Eyes down. You'll fall if you keep looking up.'</t>
         </is>
       </c>
     </row>
@@ -630,23 +614,23 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>echo1_mina_normal</t>
+          <t>echo1_sora_timing</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>ミナ:「洞窟なんだからエコーぐらいあるだろ」</t>
+          <t>ソラ:「……足音の返り、距離と合わないな」</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Mina: 'It's a cave. Echoes happen.'</t>
+          <t>Sora: '...The echo timing. It doesn't match the distance.'</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Mina: 'It's a cave. Echoes happen.'</t>
+          <t>Sora: '...The echo timing. It doesn't match the distance.'</t>
         </is>
       </c>
     </row>
@@ -658,74 +642,102 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>echo1_sora_not_normal</t>
+          <t>echo1_mina_normal</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>ソラ:「そういう話じゃない。……進もう」</t>
+          <t>ミナ:「洞窟なんだからエコーぐらいあるだろ」</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Sora: 'Not that kind of echo. ...Let's keep moving.'</t>
+          <t>Mina: 'It's a cave. Echoes happen.'</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
+          <t>Mina: 'It's a cave. Echoes happen.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>echo1_sora_not_normal</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>ソラ:「そういう話じゃない。……進もう」</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
           <t>Sora: 'Not that kind of echo. ...Let's keep moving.'</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Sora: 'Not that kind of echo. ...Let's keep moving.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
         <is>
           <t>end</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>end</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>setFlag</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>chitsii.elinikki.quest.state.echo_experiment,1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="E19" t="inlineStr">
         <is>
-          <t>fadeOut</t>
+          <t>setFlag</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.3,black</t>
+          <t>chitsii.elinikki.quest.state.echo_experiment,1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="E20" t="inlineStr">
         <is>
-          <t>setBG</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>fadeOut</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.3,black</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="E21" t="inlineStr">
+        <is>
+          <t>setBG</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="E22" t="inlineStr">
         <is>
           <t>end</t>
         </is>

</xml_diff>